<commit_message>
vault backup: 2026-05-12 23:48:30
</commit_message>
<xml_diff>
--- a/考研英语/真题统计表.xlsx
+++ b/考研英语/真题统计表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Obsidian仓库\考研\考研英语\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{271DAD85-408F-41BB-8A87-BE332D7E6066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868D2D14-6718-42D8-B5BB-CC3546D91272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.看板" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="90">
   <si>
     <t>刷题日期</t>
   </si>
@@ -1005,12 +1005,6 @@
   </si>
   <si>
     <t>人物观点题</t>
-  </si>
-  <si>
-    <t>文章提到了只能追溯一两位祖先信息。过度推断为不能
-追溯远亲祖先信息,文章完全没提到, 误选A项。
-D项正确的原因是文章首句就提到了关于精确度的问题, 为同义替换,第一句翻译错误,没看懂,而误将其排除。</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>心急了,没理解好最后一段,
@@ -1024,12 +1018,61 @@
 </t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>Text4</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">pursuit </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>和</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> interest </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>对应, 文章说重视文化追求。即鼓励文化追求。
+而我推断为文化追求享有开明的环境,也就是说重视文化追求, 不一定代表有开明的环境。</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>文章提到了只能追溯一两位祖先信息。过度推断为不能
+追溯远亲祖先信息,文章完全没提到这个信息, 误选A项。
+D项正确的原因是文章首句就提到了关于精确度的问题, 为同义替换,第一句翻译错误,没看懂,而误将其排除。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>09年的Text4太抽象了, 根本没看懂, 花了40分钟,熟词生义太多了,引申意太多了,没有知识背景很难理解。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1101,6 +1144,20 @@
       <family val="1"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1137,7 +1194,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1164,6 +1221,15 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2010,7 +2076,7 @@
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="70" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>46152</v>
       </c>
@@ -2033,15 +2099,22 @@
         <v>2</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6">
         <f>SUM(E6:H6)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" s="6">
         <f>(20-I6)/20</f>
-        <v>0.8</v>
+        <v>0.75</v>
+      </c>
+      <c r="K6">
+        <f xml:space="preserve"> 25+25+25+40</f>
+        <v>115</v>
+      </c>
+      <c r="L6" s="16" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -2081,7 +2154,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="7" width="18" style="9" customWidth="1"/>
@@ -2257,7 +2330,7 @@
       <c r="H6" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="17" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2286,7 +2359,7 @@
       <c r="H7" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="18" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2316,10 +2389,10 @@
         <v>25</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="176" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:11" ht="141" x14ac:dyDescent="0.4">
       <c r="A9" s="9" t="s">
         <v>49</v>
       </c>
@@ -2342,10 +2415,39 @@
         <v>19</v>
       </c>
       <c r="H9" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="I9" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="I9" s="15" t="s">
+    </row>
+    <row r="10" spans="1:11" ht="72" x14ac:dyDescent="0.4">
+      <c r="A10" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="9">
+        <v>2009</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>86</v>
+      </c>
+      <c r="D10" s="9">
+        <v>36</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>